<commit_message>
more done (added orbital filing and n=)
</commit_message>
<xml_diff>
--- a/OER/Volcano_Charter/CDG790-z.xlsx
+++ b/OER/Volcano_Charter/CDG790-z.xlsx
@@ -6,8 +6,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="100mv" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5mv" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="100mv (1-2-3)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5mv (4-2-1)" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
@@ -19086,7 +19086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19097,30 +19097,40 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>n=</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Orbital Filling</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Avg j at 1.75 V (mA/cm²)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Std j at 1.75 V</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Avg E at 0.5 mA/cm² (V)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Std E at 0.5 mA/cm²</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Avg E at 1.0 mA/cm² (V)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Std E at 1.0 mA/cm²</t>
         </is>
@@ -19129,50 +19139,62 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>100mv</t>
+          <t>100mv (1-2-3)</t>
         </is>
       </c>
       <c r="B2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="D2" t="n">
         <v>0.8517452220782755</v>
       </c>
-      <c r="C2" t="n">
+      <c r="E2" t="n">
         <v>0.03691795918297232</v>
       </c>
-      <c r="D2" t="n">
+      <c r="F2" t="n">
         <v>1.712254577788928</v>
       </c>
-      <c r="E2" t="n">
+      <c r="G2" t="n">
         <v>0.002227375768281577</v>
       </c>
-      <c r="F2" t="n">
+      <c r="H2" t="n">
         <v>1.761926145239876</v>
       </c>
-      <c r="G2" t="n">
+      <c r="I2" t="n">
         <v>0.003285201707157113</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>5mv</t>
+          <t>5mv (4-2-1)</t>
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="n">
+        <v>15</v>
+      </c>
+      <c r="D3" t="n">
         <v>0.319823818431964</v>
       </c>
-      <c r="C3" t="n">
+      <c r="E3" t="n">
         <v>0.02933376093155236</v>
       </c>
-      <c r="D3" t="n">
+      <c r="F3" t="n">
         <v>1.781896954590296</v>
       </c>
-      <c r="E3" t="n">
+      <c r="G3" t="n">
         <v>0.008584834295337742</v>
       </c>
-      <c r="F3" t="n">
+      <c r="H3" t="n">
         <v>1.843448653256587</v>
       </c>
-      <c r="G3" t="n">
+      <c r="I3" t="n">
         <v>0.01223768116145332</v>
       </c>
     </row>

</xml_diff>